<commit_message>
chore: Update appeals_monitor_feedback.xlsx with new data
</commit_message>
<xml_diff>
--- a/kobo/appeals_monitor_feedback.xlsx
+++ b/kobo/appeals_monitor_feedback.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rodekruis-my.sharepoint.com/personal/jmargutti_redcross_nl/Documents/Rode Kruis/510/appeals-monitor/kobo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_96B1FF8C77A348DFF8FA0826381CBB28B6AD0C6F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A39A0F3-D8BF-41D5-A5E1-004B0FAA4996}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_96B1FF8C77A348DFF8FA0826381CBB28B6AD0C6F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6524AF87-AB4F-402F-90E9-638B5D474D7D}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -694,13 +694,13 @@
     <t>English (en)</t>
   </si>
   <si>
+    <t>Comparing budgets, targets or activities against other operations</t>
+  </si>
+  <si>
     <t>**Appeals Monitor - your feedback**
-The Appeals Monitor emails you a short summary every time a new IFRC appeal document (a DREF operation, emergency appeal, operational strategy or anticipatory-action activation) is published in one of the sectors you follow.
+The Appeals Monitor emails you a short summary every time a new IFRC appeal document (a DREF operation, emergency appeal, operational strategy or anticipatory-action activation) is published and matches one of the sectors you follow.
 We would like to know whether it is actually useful to you, and what we should build next. This takes about 5 minutes. All questions are optional unless marked.
 Your answers will only be used to improve the service.</t>
-  </si>
-  <si>
-    <t>Comparing budgets, targets or activities against other operations</t>
   </si>
 </sst>
 </file>
@@ -762,6 +762,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1110,7 +1114,7 @@
         <v>130</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
@@ -1892,7 +1896,7 @@
         <v>38</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">

</xml_diff>

<commit_message>
refactor: remove retry logic for bad request in form deployment
</commit_message>
<xml_diff>
--- a/kobo/appeals_monitor_feedback.xlsx
+++ b/kobo/appeals_monitor_feedback.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JMargutti\OneDrive - Rode Kruis\Rode Kruis\510\appeals-monitor\kobo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06651E35-F0C9-494A-B936-CC03EE2A41B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87417E9B-C586-4DCA-9053-6DFFA9C516BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="205">
   <si>
     <t>list_name</t>
   </si>
@@ -571,15 +571,6 @@
   </si>
   <si>
     <t>selected(${preferred_channels}, 'other')</t>
-  </si>
-  <si>
-    <t>doctypes_other</t>
-  </si>
-  <si>
-    <t>Please specify the other documents</t>
-  </si>
-  <si>
-    <t>selected(${extra_doctypes}, 'other')</t>
   </si>
   <si>
     <t>missing_content</t>
@@ -998,7 +989,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1059,7 +1050,7 @@
         <v>113</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
@@ -1523,16 +1514,18 @@
       <c r="C25" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="D25" s="2"/>
+      <c r="D25" s="2" t="s">
+        <v>185</v>
+      </c>
       <c r="E25" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>185</v>
-      </c>
+      <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
+      <c r="I25" s="2" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="2" t="s">
@@ -1544,9 +1537,7 @@
       <c r="C26" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>188</v>
-      </c>
+      <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
         <v>111</v>
       </c>
@@ -1557,60 +1548,39 @@
         <v>152</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>190</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="C27" s="2"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="2" t="s">
-        <v>111</v>
-      </c>
+      <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="2" t="s">
-        <v>152</v>
-      </c>
+      <c r="I27" s="2"/>
     </row>
     <row r="28" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="2" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C28" s="2"/>
+        <v>188</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>189</v>
+      </c>
       <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
+      <c r="E28" s="2" t="s">
+        <v>111</v>
+      </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1822,7 +1792,7 @@
         <v>38</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
@@ -1830,10 +1800,10 @@
         <v>27</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
@@ -2020,7 +1990,7 @@
         <v>74</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.55000000000000004">
@@ -2241,36 +2211,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>